<commit_message>
rules v1.3: 4 mm between overlay facades; GibLab sizes are finished sizes
Decisions of the product owner from a real order (GibLab):
- gap between adjacent overlay facades 4 mm (horizontal and vertical);
- facade edging stays KR08 0.8 mm;
- GibLab part sizes are finished sizes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAoMGr6KDaXSM8LT5Nrkkp
</commit_message>
<xml_diff>
--- a/docs/Elvin_pytannia_tehnologu.xlsx
+++ b/docs/Elvin_pytannia_tehnologu.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="218">
   <si>
     <t xml:space="preserve">Elvin — питання технологу</t>
   </si>
@@ -615,27 +615,33 @@
     <t xml:space="preserve">Розміри фасадів.</t>
   </si>
   <si>
-    <t xml:space="preserve">Верх 3, низ 3, боки 2, між фасадами 2 мм</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 / 3 / 2 / 2</t>
+    <t xml:space="preserve">Верх 3, низ 3, боки 2, між фасадами 4 мм (по горизонталі й вертикалі)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 / 3 / 2 / 4</t>
   </si>
   <si>
     <t xml:space="preserve">Користувач (чат)</t>
   </si>
   <si>
+    <t xml:space="preserve">16.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Між фасадами 4 мм — за реальним замовленням (GibLab), підтверджено 16.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Максимальний розмір листа ХДФ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2800 × 2070 мм</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2800 × 2070</t>
+  </si>
+  <si>
     <t xml:space="preserve">15.10.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Максимальний розмір листа ХДФ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2800 × 2070 мм</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2800 × 2070</t>
-  </si>
-  <si>
     <t xml:space="preserve">Накладна ХДФ: один лист чи окремі по секціях?</t>
   </si>
   <si>
@@ -652,6 +658,27 @@
   </si>
   <si>
     <t xml:space="preserve">Як на фабриці: ST_L, ST_R, ST_SR, DNO, KR, POLKA, TYL, COKOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Розміри деталей у GibLab — готові (з кромкою) чи заготовки?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Звірка Elvin з GibLab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Готові розміри деталей</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кромка фасадів: ABS 1 мм (як у GibLab) чи KR08 0,8 мм?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кромкування фасадів.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Правила: KR08 0,8 мм.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Лишаємо KR08 0,8 мм; змінюється в 1 клік</t>
   </si>
 </sst>
 </file>
@@ -815,16 +842,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -836,15 +867,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -852,7 +883,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -860,7 +891,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -868,11 +899,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1188,82 +1219,82 @@
   <dimension ref="B2:C13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="90"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3" t="s">
+    <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="3" t="s">
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="3" t="s">
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="3" t="s">
+    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="3" t="s">
+    <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1286,335 +1317,335 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A4)</f>
         <v>6</v>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>6</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
         <v>0</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A5)</f>
         <v>5</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>5</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
         <v>0</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A6)</f>
         <v>3</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A6,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>3</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A6,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A6,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A6,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
         <v>0</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A6,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A7)</f>
         <v>17</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>15</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
         <v>2</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A8)</f>
         <v>5</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A8,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>5</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A8,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A8,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A8,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
         <v>0</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A8,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A9)</f>
         <v>5</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A9,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>5</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A9,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A9,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A9,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
         <v>0</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A9,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A10)</f>
-        <v>4</v>
-      </c>
-      <c r="C10" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>3</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>1</v>
-      </c>
-      <c r="G10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A11)</f>
         <v>3</v>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A11,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>3</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A11,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A11,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A11,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
         <v>0</v>
       </c>
-      <c r="G11" s="10" t="n">
+      <c r="G11" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A11,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A12)</f>
-        <v>5</v>
-      </c>
-      <c r="C12" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A12,Питання!$L$2:$L$200,"Відкрито")</f>
         <v>4</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A12,Питання!$L$2:$L$200,"Відповідь отримано")</f>
         <v>0</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A12,Питання!$L$2:$L$200,"Потрібен скрипт BAZIS")</f>
         <v>0</v>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A12,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>1</v>
-      </c>
-      <c r="G12" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A12,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <f aca="false">SUM(B4:B12)</f>
-        <v>53</v>
-      </c>
-      <c r="C13" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="C13" s="13" t="n">
         <f aca="false">SUM(C4:C12)</f>
         <v>49</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">SUM(D4:D12)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">SUM(E4:E12)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">SUM(F4:F12)</f>
-        <v>4</v>
-      </c>
-      <c r="G13" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="13" t="n">
         <f aca="false">SUM(G4:G12)</f>
         <v>9</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="15" t="n">
         <f aca="false">IF(B13=0,0,F13/B13)</f>
-        <v>0.0754716981132075</v>
+        <v>0.109090909090909</v>
       </c>
     </row>
   </sheetData>
@@ -1636,2012 +1667,2048 @@
   <dimension ref="A1:M74"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="15" t="n">
+    <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M2" s="16"/>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="n">
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" s="17"/>
+    </row>
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M3" s="16"/>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="n">
+      <c r="G3" s="16"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M3" s="17"/>
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M4" s="16"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="n">
+      <c r="G4" s="16"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M4" s="17"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M5" s="16"/>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="n">
+      <c r="G5" s="16"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M6" s="16"/>
-    </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="n">
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" s="17"/>
+    </row>
+    <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M7" s="16"/>
-    </row>
-    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="n">
+      <c r="G7" s="16"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M7" s="17"/>
+    </row>
+    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M8" s="16"/>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="n">
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M8" s="17"/>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M9" s="16"/>
-    </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="n">
+      <c r="G9" s="16"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M9" s="17"/>
+    </row>
+    <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M10" s="16"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="n">
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M10" s="17"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M11" s="16"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="n">
+      <c r="G11" s="16"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M11" s="17"/>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G12" s="15"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M12" s="16"/>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="n">
+      <c r="G12" s="16"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M12" s="17"/>
+    </row>
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="n">
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M13" s="17"/>
+    </row>
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G14" s="15"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="n">
+      <c r="G14" s="16"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M14" s="17"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M15" s="16"/>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="n">
+      <c r="G15" s="16"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M15" s="17"/>
+    </row>
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="F16" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="16" t="s">
+      <c r="G16" s="16"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M16" s="17" t="s">
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M16" s="18" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="n">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G17" s="15"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M17" s="16"/>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="n">
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M17" s="17"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="E18" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="F18" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="G18" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M18" s="16"/>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="n">
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M18" s="17"/>
+    </row>
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="E19" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="F19" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M19" s="16"/>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="n">
+      <c r="G19" s="16"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M19" s="17"/>
+    </row>
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="F20" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="G20" s="15"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M20" s="16"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="n">
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M20" s="17"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="F21" s="15" t="s">
+      <c r="F21" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="G21" s="15" t="s">
+      <c r="G21" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M21" s="16"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="15" t="s">
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M21" s="17"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="F22" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="G22" s="15"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M22" s="16"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="n">
+      <c r="G22" s="16"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M22" s="17"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="F23" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G23" s="15"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M23" s="16"/>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="n">
+      <c r="G23" s="16"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M23" s="17"/>
+    </row>
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="16" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="F24" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="G24" s="15"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M24" s="16"/>
-    </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="n">
+      <c r="G24" s="16"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M24" s="17"/>
+    </row>
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F25" s="15" t="s">
+      <c r="F25" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G25" s="15"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16" t="s">
+      <c r="G25" s="16"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M25" s="17" t="s">
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M25" s="18" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="n">
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="E26" s="15" t="s">
+      <c r="E26" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F26" s="15" t="s">
+      <c r="F26" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G26" s="15"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="16"/>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M26" s="16"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="n">
+      <c r="G26" s="16"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M26" s="17"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="E27" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="F27" s="15" t="s">
+      <c r="F27" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G27" s="15"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M27" s="16"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="n">
+      <c r="G27" s="16"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M27" s="17"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="F28" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G28" s="15"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M28" s="16"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="n">
+      <c r="G28" s="16"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M28" s="17"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="E29" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="F29" s="15" t="s">
+      <c r="F29" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="G29" s="15"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M29" s="16"/>
-    </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="n">
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M29" s="17"/>
+    </row>
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="15" t="s">
+      <c r="B30" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="E30" s="15" t="s">
+      <c r="E30" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="F30" s="15" t="s">
+      <c r="F30" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="G30" s="15" t="s">
+      <c r="G30" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M30" s="16"/>
-    </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="n">
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M30" s="17"/>
+    </row>
+    <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="E31" s="15" t="s">
+      <c r="E31" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F31" s="15" t="s">
+      <c r="F31" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="G31" s="15"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M31" s="16"/>
-    </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="n">
+      <c r="G31" s="16"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
+      <c r="K31" s="17"/>
+      <c r="L31" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M31" s="17"/>
+    </row>
+    <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="B32" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="C32" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="E32" s="15" t="s">
+      <c r="E32" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="F32" s="15" t="s">
+      <c r="F32" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="G32" s="15"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M32" s="16"/>
-    </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="n">
+      <c r="G32" s="16"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M32" s="17"/>
+    </row>
+    <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="16" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D33" s="15" t="s">
+      <c r="D33" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="E33" s="15" t="s">
+      <c r="E33" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F33" s="15" t="s">
+      <c r="F33" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G33" s="15"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M33" s="16"/>
-    </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15" t="n">
+      <c r="G33" s="16"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+      <c r="L33" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M33" s="17"/>
+    </row>
+    <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="15" t="s">
+      <c r="B34" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D34" s="15" t="s">
+      <c r="D34" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="E34" s="15" t="s">
+      <c r="E34" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="F34" s="15" t="s">
+      <c r="F34" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="G34" s="15"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M34" s="16"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="n">
+      <c r="G34" s="16"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+      <c r="L34" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M34" s="17"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D35" s="15" t="s">
+      <c r="D35" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="E35" s="15" t="s">
+      <c r="E35" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="F35" s="15" t="s">
+      <c r="F35" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G35" s="15"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M35" s="16"/>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15" t="n">
+      <c r="G35" s="16"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+      <c r="L35" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M35" s="17"/>
+    </row>
+    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="B36" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C36" s="15" t="s">
+      <c r="C36" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D36" s="15" t="s">
+      <c r="D36" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="E36" s="15" t="s">
+      <c r="E36" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="F36" s="15" t="s">
+      <c r="F36" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="G36" s="15"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="16"/>
-      <c r="J36" s="16"/>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M36" s="16"/>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="n">
+      <c r="G36" s="16"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+      <c r="L36" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M36" s="17"/>
+    </row>
+    <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C37" s="15" t="s">
+      <c r="C37" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D37" s="15" t="s">
+      <c r="D37" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E37" s="15" t="s">
+      <c r="E37" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="F37" s="15" t="s">
+      <c r="F37" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="G37" s="15" t="s">
+      <c r="G37" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="H37" s="16"/>
-      <c r="I37" s="16"/>
-      <c r="J37" s="16"/>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M37" s="16"/>
-    </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="n">
+      <c r="H37" s="17"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M37" s="17"/>
+    </row>
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="16" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C38" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D38" s="15" t="s">
+      <c r="D38" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="E38" s="15" t="s">
+      <c r="E38" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="F38" s="15" t="s">
+      <c r="F38" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="G38" s="15" t="s">
+      <c r="G38" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16"/>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M38" s="16"/>
-    </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="n">
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M38" s="17"/>
+    </row>
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="15" t="s">
+      <c r="B39" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C39" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D39" s="15" t="s">
+      <c r="D39" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="E39" s="15" t="s">
+      <c r="E39" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="F39" s="15" t="s">
+      <c r="F39" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="G39" s="15" t="s">
+      <c r="G39" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="H39" s="16"/>
-      <c r="I39" s="16"/>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M39" s="16"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="n">
+      <c r="H39" s="17"/>
+      <c r="I39" s="17"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M39" s="17"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="15" t="s">
+      <c r="B40" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C40" s="15" t="s">
+      <c r="C40" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D40" s="15" t="s">
+      <c r="D40" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="E40" s="15" t="s">
+      <c r="E40" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="F40" s="15" t="s">
+      <c r="F40" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="G40" s="15"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="16"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M40" s="16"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="15" t="n">
+      <c r="G40" s="16"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="17"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+      <c r="L40" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M40" s="17"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="15" t="s">
+      <c r="B41" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C41" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D41" s="15" t="s">
+      <c r="D41" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="E41" s="15" t="s">
+      <c r="E41" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="F41" s="15" t="s">
+      <c r="F41" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="G41" s="15"/>
-      <c r="H41" s="16"/>
-      <c r="I41" s="16" t="s">
+      <c r="G41" s="16"/>
+      <c r="H41" s="17"/>
+      <c r="I41" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="J41" s="16"/>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M41" s="17" t="s">
+      <c r="J41" s="17"/>
+      <c r="K41" s="17"/>
+      <c r="L41" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M41" s="18" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="n">
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="15" t="s">
+      <c r="B42" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="15" t="s">
+      <c r="C42" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="E42" s="15" t="s">
+      <c r="E42" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="F42" s="15" t="s">
+      <c r="F42" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="G42" s="15"/>
-      <c r="H42" s="16"/>
-      <c r="I42" s="16"/>
-      <c r="J42" s="16"/>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M42" s="16"/>
-    </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="n">
+      <c r="G42" s="16"/>
+      <c r="H42" s="17"/>
+      <c r="I42" s="17"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="17"/>
+      <c r="L42" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M42" s="17"/>
+    </row>
+    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="16" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="15" t="s">
+      <c r="B43" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C43" s="15" t="s">
+      <c r="C43" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D43" s="15" t="s">
+      <c r="D43" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="E43" s="15" t="s">
+      <c r="E43" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="F43" s="15" t="s">
+      <c r="F43" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G43" s="15"/>
-      <c r="H43" s="16"/>
-      <c r="I43" s="16"/>
-      <c r="J43" s="16"/>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M43" s="16"/>
-    </row>
-    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="n">
+      <c r="G43" s="16"/>
+      <c r="H43" s="17"/>
+      <c r="I43" s="17"/>
+      <c r="J43" s="17"/>
+      <c r="K43" s="17"/>
+      <c r="L43" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M43" s="17"/>
+    </row>
+    <row r="44" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="16" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="15" t="s">
+      <c r="B44" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C44" s="15" t="s">
+      <c r="C44" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D44" s="15" t="s">
+      <c r="D44" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="E44" s="15" t="s">
+      <c r="E44" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="F44" s="15" t="s">
+      <c r="F44" s="16" t="s">
         <v>175</v>
       </c>
-      <c r="G44" s="15" t="s">
+      <c r="G44" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="H44" s="16"/>
-      <c r="I44" s="16"/>
-      <c r="J44" s="16"/>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M44" s="16"/>
-    </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="n">
+      <c r="H44" s="17"/>
+      <c r="I44" s="17"/>
+      <c r="J44" s="17"/>
+      <c r="K44" s="17"/>
+      <c r="L44" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M44" s="17"/>
+    </row>
+    <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="15" t="s">
+      <c r="B45" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C45" s="15" t="s">
+      <c r="C45" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D45" s="15" t="s">
+      <c r="D45" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="E45" s="15" t="s">
+      <c r="E45" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="F45" s="15" t="s">
+      <c r="F45" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="G45" s="15"/>
-      <c r="H45" s="16"/>
-      <c r="I45" s="16"/>
-      <c r="J45" s="16"/>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M45" s="16"/>
-    </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="n">
+      <c r="G45" s="16"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M45" s="17"/>
+    </row>
+    <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="15" t="s">
+      <c r="B46" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C46" s="15" t="s">
+      <c r="C46" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D46" s="15" t="s">
+      <c r="D46" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="E46" s="15" t="s">
+      <c r="E46" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F46" s="15" t="s">
+      <c r="F46" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="G46" s="15"/>
-      <c r="H46" s="16"/>
-      <c r="I46" s="16"/>
-      <c r="J46" s="16"/>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M46" s="16"/>
-    </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="n">
+      <c r="G46" s="16"/>
+      <c r="H46" s="17"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="17"/>
+      <c r="K46" s="17"/>
+      <c r="L46" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M46" s="17"/>
+    </row>
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="16" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C47" s="15" t="s">
+      <c r="C47" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D47" s="15" t="s">
+      <c r="D47" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="E47" s="15" t="s">
+      <c r="E47" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F47" s="15" t="s">
+      <c r="F47" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="G47" s="15"/>
-      <c r="H47" s="16"/>
-      <c r="I47" s="16"/>
-      <c r="J47" s="16"/>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M47" s="16"/>
-    </row>
-    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="n">
+      <c r="G47" s="16"/>
+      <c r="H47" s="17"/>
+      <c r="I47" s="17"/>
+      <c r="J47" s="17"/>
+      <c r="K47" s="17"/>
+      <c r="L47" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M47" s="17"/>
+    </row>
+    <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="16" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="B48" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C48" s="15" t="s">
+      <c r="C48" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="15" t="s">
+      <c r="D48" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="E48" s="15" t="s">
+      <c r="E48" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="F48" s="15" t="s">
+      <c r="F48" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="G48" s="15"/>
-      <c r="H48" s="16"/>
-      <c r="I48" s="16"/>
-      <c r="J48" s="16"/>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M48" s="16"/>
-    </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="n">
+      <c r="G48" s="16"/>
+      <c r="H48" s="17"/>
+      <c r="I48" s="17"/>
+      <c r="J48" s="17"/>
+      <c r="K48" s="17"/>
+      <c r="L48" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M48" s="17"/>
+    </row>
+    <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="16" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="15" t="s">
+      <c r="B49" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C49" s="15" t="s">
+      <c r="C49" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D49" s="15" t="s">
+      <c r="D49" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="E49" s="15" t="s">
+      <c r="E49" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="F49" s="15" t="s">
+      <c r="F49" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="G49" s="15"/>
-      <c r="H49" s="16"/>
-      <c r="I49" s="16"/>
-      <c r="J49" s="16"/>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M49" s="16"/>
-    </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="n">
+      <c r="G49" s="16"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+      <c r="J49" s="17"/>
+      <c r="K49" s="17"/>
+      <c r="L49" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M49" s="17"/>
+    </row>
+    <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="16" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B50" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C50" s="15" t="s">
+      <c r="C50" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D50" s="15" t="s">
+      <c r="D50" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="E50" s="15" t="s">
+      <c r="E50" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="F50" s="15" t="s">
+      <c r="F50" s="16" t="s">
         <v>193</v>
       </c>
-      <c r="G50" s="15"/>
-      <c r="H50" s="16"/>
-      <c r="I50" s="16"/>
-      <c r="J50" s="16"/>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M50" s="16"/>
-    </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="n">
+      <c r="G50" s="16"/>
+      <c r="H50" s="17"/>
+      <c r="I50" s="17"/>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
+      <c r="L50" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M50" s="17"/>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="15" t="s">
+      <c r="B51" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C51" s="15" t="s">
+      <c r="C51" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D51" s="15" t="s">
+      <c r="D51" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="E51" s="15" t="s">
+      <c r="E51" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="F51" s="15"/>
-      <c r="G51" s="15"/>
-      <c r="H51" s="16" t="s">
+      <c r="F51" s="16"/>
+      <c r="G51" s="16"/>
+      <c r="H51" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="I51" s="16" t="s">
+      <c r="I51" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="J51" s="16" t="s">
+      <c r="J51" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="K51" s="16" t="s">
+      <c r="K51" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="L51" s="16" t="s">
+      <c r="L51" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="M51" s="16"/>
-    </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="n">
+      <c r="M51" s="17" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="16" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="15" t="s">
+      <c r="B52" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C52" s="15" t="s">
+      <c r="C52" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D52" s="15" t="s">
-        <v>200</v>
-      </c>
-      <c r="E52" s="15" t="s">
+      <c r="D52" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="E52" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="F52" s="15"/>
-      <c r="G52" s="15"/>
-      <c r="H52" s="16" t="s">
-        <v>201</v>
-      </c>
-      <c r="I52" s="16" t="s">
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="J52" s="16" t="s">
+      <c r="I52" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="J52" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="K52" s="16" t="s">
+      <c r="K52" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="L52" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="M52" s="17"/>
+    </row>
+    <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="16" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D53" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="E53" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="F53" s="16"/>
+      <c r="G53" s="16"/>
+      <c r="H53" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="I53" s="17"/>
+      <c r="J53" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="K53" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="L53" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="M53" s="17"/>
+    </row>
+    <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="16" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C54" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D54" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="E54" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="F54" s="16"/>
+      <c r="G54" s="16"/>
+      <c r="H54" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="I54" s="17"/>
+      <c r="J54" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="K54" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="L54" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="M54" s="17"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="16" t="n">
+        <f aca="false">IF(D55="","",ROW()-1)</f>
+        <v>54</v>
+      </c>
+      <c r="B55" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C55" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D55" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="E55" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+      <c r="H55" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="I55" s="17"/>
+      <c r="J55" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="K55" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="L52" s="16" t="s">
+      <c r="L55" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="M52" s="16"/>
-    </row>
-    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C53" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D53" s="15" t="s">
-        <v>203</v>
-      </c>
-      <c r="E53" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="16" t="s">
-        <v>205</v>
-      </c>
-      <c r="I53" s="16"/>
-      <c r="J53" s="16" t="s">
+      <c r="M55" s="17"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="16" t="n">
+        <f aca="false">IF(D56="","",ROW()-1)</f>
+        <v>55</v>
+      </c>
+      <c r="B56" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C56" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="D56" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="E56" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="F56" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="G56" s="16"/>
+      <c r="H56" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="I56" s="17"/>
+      <c r="J56" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="K53" s="16" t="s">
+      <c r="K56" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="L53" s="16" t="s">
+      <c r="L56" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="M53" s="16"/>
-    </row>
-    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C54" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D54" s="15" t="s">
-        <v>206</v>
-      </c>
-      <c r="E54" s="15" t="s">
-        <v>207</v>
-      </c>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="I54" s="16"/>
-      <c r="J54" s="16" t="s">
-        <v>198</v>
-      </c>
-      <c r="K54" s="16" t="s">
-        <v>199</v>
-      </c>
-      <c r="L54" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="M54" s="16"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="15" t="str">
-        <f aca="false">IF(D55="","",ROW()-1)</f>
-        <v/>
-      </c>
-      <c r="B55" s="16"/>
-      <c r="C55" s="16"/>
-      <c r="D55" s="16"/>
-      <c r="E55" s="15"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="15"/>
-      <c r="H55" s="16"/>
-      <c r="I55" s="16"/>
-      <c r="J55" s="16"/>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
-      <c r="M55" s="16"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="15" t="str">
-        <f aca="false">IF(D56="","",ROW()-1)</f>
-        <v/>
-      </c>
-      <c r="B56" s="16"/>
-      <c r="C56" s="16"/>
-      <c r="D56" s="16"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
-      <c r="H56" s="16"/>
-      <c r="I56" s="16"/>
-      <c r="J56" s="16"/>
-      <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
-      <c r="M56" s="16"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="15" t="str">
+      <c r="M56" s="17"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="16" t="str">
         <f aca="false">IF(D57="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B57" s="16"/>
-      <c r="C57" s="16"/>
-      <c r="D57" s="16"/>
-      <c r="E57" s="15"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
-      <c r="H57" s="16"/>
-      <c r="I57" s="16"/>
-      <c r="J57" s="16"/>
-      <c r="K57" s="16"/>
-      <c r="L57" s="16"/>
-      <c r="M57" s="16"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="15" t="str">
+      <c r="B57" s="17"/>
+      <c r="C57" s="17"/>
+      <c r="D57" s="17"/>
+      <c r="E57" s="16"/>
+      <c r="F57" s="16"/>
+      <c r="G57" s="16"/>
+      <c r="H57" s="17"/>
+      <c r="I57" s="17"/>
+      <c r="J57" s="17"/>
+      <c r="K57" s="17"/>
+      <c r="L57" s="17"/>
+      <c r="M57" s="17"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="16" t="str">
         <f aca="false">IF(D58="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B58" s="16"/>
-      <c r="C58" s="16"/>
-      <c r="D58" s="16"/>
-      <c r="E58" s="15"/>
-      <c r="F58" s="15"/>
-      <c r="G58" s="15"/>
-      <c r="H58" s="16"/>
-      <c r="I58" s="16"/>
-      <c r="J58" s="16"/>
-      <c r="K58" s="16"/>
-      <c r="L58" s="16"/>
-      <c r="M58" s="16"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="15" t="str">
+      <c r="B58" s="17"/>
+      <c r="C58" s="17"/>
+      <c r="D58" s="17"/>
+      <c r="E58" s="16"/>
+      <c r="F58" s="16"/>
+      <c r="G58" s="16"/>
+      <c r="H58" s="17"/>
+      <c r="I58" s="17"/>
+      <c r="J58" s="17"/>
+      <c r="K58" s="17"/>
+      <c r="L58" s="17"/>
+      <c r="M58" s="17"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="16" t="str">
         <f aca="false">IF(D59="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B59" s="16"/>
-      <c r="C59" s="16"/>
-      <c r="D59" s="16"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
-      <c r="H59" s="16"/>
-      <c r="I59" s="16"/>
-      <c r="J59" s="16"/>
-      <c r="K59" s="16"/>
-      <c r="L59" s="16"/>
-      <c r="M59" s="16"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="15" t="str">
+      <c r="B59" s="17"/>
+      <c r="C59" s="17"/>
+      <c r="D59" s="17"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
+      <c r="H59" s="17"/>
+      <c r="I59" s="17"/>
+      <c r="J59" s="17"/>
+      <c r="K59" s="17"/>
+      <c r="L59" s="17"/>
+      <c r="M59" s="17"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="16" t="str">
         <f aca="false">IF(D60="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B60" s="16"/>
-      <c r="C60" s="16"/>
-      <c r="D60" s="16"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="15"/>
-      <c r="G60" s="15"/>
-      <c r="H60" s="16"/>
-      <c r="I60" s="16"/>
-      <c r="J60" s="16"/>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="15" t="str">
+      <c r="B60" s="17"/>
+      <c r="C60" s="17"/>
+      <c r="D60" s="17"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="16"/>
+      <c r="H60" s="17"/>
+      <c r="I60" s="17"/>
+      <c r="J60" s="17"/>
+      <c r="K60" s="17"/>
+      <c r="L60" s="17"/>
+      <c r="M60" s="17"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="16" t="str">
         <f aca="false">IF(D61="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B61" s="16"/>
-      <c r="C61" s="16"/>
-      <c r="D61" s="16"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="16"/>
-      <c r="I61" s="16"/>
-      <c r="J61" s="16"/>
-      <c r="K61" s="16"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="15" t="str">
+      <c r="B61" s="17"/>
+      <c r="C61" s="17"/>
+      <c r="D61" s="17"/>
+      <c r="E61" s="16"/>
+      <c r="F61" s="16"/>
+      <c r="G61" s="16"/>
+      <c r="H61" s="17"/>
+      <c r="I61" s="17"/>
+      <c r="J61" s="17"/>
+      <c r="K61" s="17"/>
+      <c r="L61" s="17"/>
+      <c r="M61" s="17"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="16" t="str">
         <f aca="false">IF(D62="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B62" s="16"/>
-      <c r="C62" s="16"/>
-      <c r="D62" s="16"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="15"/>
-      <c r="G62" s="15"/>
-      <c r="H62" s="16"/>
-      <c r="I62" s="16"/>
-      <c r="J62" s="16"/>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16"/>
-      <c r="M62" s="16"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="15" t="str">
+      <c r="B62" s="17"/>
+      <c r="C62" s="17"/>
+      <c r="D62" s="17"/>
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+      <c r="G62" s="16"/>
+      <c r="H62" s="17"/>
+      <c r="I62" s="17"/>
+      <c r="J62" s="17"/>
+      <c r="K62" s="17"/>
+      <c r="L62" s="17"/>
+      <c r="M62" s="17"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="16" t="str">
         <f aca="false">IF(D63="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B63" s="16"/>
-      <c r="C63" s="16"/>
-      <c r="D63" s="16"/>
-      <c r="E63" s="15"/>
-      <c r="F63" s="15"/>
-      <c r="G63" s="15"/>
-      <c r="H63" s="16"/>
-      <c r="I63" s="16"/>
-      <c r="J63" s="16"/>
-      <c r="K63" s="16"/>
-      <c r="L63" s="16"/>
-      <c r="M63" s="16"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="15" t="str">
+      <c r="B63" s="17"/>
+      <c r="C63" s="17"/>
+      <c r="D63" s="17"/>
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+      <c r="G63" s="16"/>
+      <c r="H63" s="17"/>
+      <c r="I63" s="17"/>
+      <c r="J63" s="17"/>
+      <c r="K63" s="17"/>
+      <c r="L63" s="17"/>
+      <c r="M63" s="17"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="16" t="str">
         <f aca="false">IF(D64="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B64" s="16"/>
-      <c r="C64" s="16"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="15"/>
-      <c r="F64" s="15"/>
-      <c r="G64" s="15"/>
-      <c r="H64" s="16"/>
-      <c r="I64" s="16"/>
-      <c r="J64" s="16"/>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="15" t="str">
+      <c r="B64" s="17"/>
+      <c r="C64" s="17"/>
+      <c r="D64" s="17"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="17"/>
+      <c r="I64" s="17"/>
+      <c r="J64" s="17"/>
+      <c r="K64" s="17"/>
+      <c r="L64" s="17"/>
+      <c r="M64" s="17"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="16" t="str">
         <f aca="false">IF(D65="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B65" s="16"/>
-      <c r="C65" s="16"/>
-      <c r="D65" s="16"/>
-      <c r="E65" s="15"/>
-      <c r="F65" s="15"/>
-      <c r="G65" s="15"/>
-      <c r="H65" s="16"/>
-      <c r="I65" s="16"/>
-      <c r="J65" s="16"/>
-      <c r="K65" s="16"/>
-      <c r="L65" s="16"/>
-      <c r="M65" s="16"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="15" t="str">
+      <c r="B65" s="17"/>
+      <c r="C65" s="17"/>
+      <c r="D65" s="17"/>
+      <c r="E65" s="16"/>
+      <c r="F65" s="16"/>
+      <c r="G65" s="16"/>
+      <c r="H65" s="17"/>
+      <c r="I65" s="17"/>
+      <c r="J65" s="17"/>
+      <c r="K65" s="17"/>
+      <c r="L65" s="17"/>
+      <c r="M65" s="17"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="16" t="str">
         <f aca="false">IF(D66="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B66" s="16"/>
-      <c r="C66" s="16"/>
-      <c r="D66" s="16"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="15"/>
-      <c r="G66" s="15"/>
-      <c r="H66" s="16"/>
-      <c r="I66" s="16"/>
-      <c r="J66" s="16"/>
-      <c r="K66" s="16"/>
-      <c r="L66" s="16"/>
-      <c r="M66" s="16"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="15" t="str">
+      <c r="B66" s="17"/>
+      <c r="C66" s="17"/>
+      <c r="D66" s="17"/>
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+      <c r="G66" s="16"/>
+      <c r="H66" s="17"/>
+      <c r="I66" s="17"/>
+      <c r="J66" s="17"/>
+      <c r="K66" s="17"/>
+      <c r="L66" s="17"/>
+      <c r="M66" s="17"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="16" t="str">
         <f aca="false">IF(D67="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B67" s="16"/>
-      <c r="C67" s="16"/>
-      <c r="D67" s="16"/>
-      <c r="E67" s="15"/>
-      <c r="F67" s="15"/>
-      <c r="G67" s="15"/>
-      <c r="H67" s="16"/>
-      <c r="I67" s="16"/>
-      <c r="J67" s="16"/>
-      <c r="K67" s="16"/>
-      <c r="L67" s="16"/>
-      <c r="M67" s="16"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="15" t="str">
+      <c r="B67" s="17"/>
+      <c r="C67" s="17"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16"/>
+      <c r="H67" s="17"/>
+      <c r="I67" s="17"/>
+      <c r="J67" s="17"/>
+      <c r="K67" s="17"/>
+      <c r="L67" s="17"/>
+      <c r="M67" s="17"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="16" t="str">
         <f aca="false">IF(D68="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B68" s="16"/>
-      <c r="C68" s="16"/>
-      <c r="D68" s="16"/>
-      <c r="E68" s="15"/>
-      <c r="F68" s="15"/>
-      <c r="G68" s="15"/>
-      <c r="H68" s="16"/>
-      <c r="I68" s="16"/>
-      <c r="J68" s="16"/>
-      <c r="K68" s="16"/>
-      <c r="L68" s="16"/>
-      <c r="M68" s="16"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="15" t="str">
+      <c r="B68" s="17"/>
+      <c r="C68" s="17"/>
+      <c r="D68" s="17"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
+      <c r="H68" s="17"/>
+      <c r="I68" s="17"/>
+      <c r="J68" s="17"/>
+      <c r="K68" s="17"/>
+      <c r="L68" s="17"/>
+      <c r="M68" s="17"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="16" t="str">
         <f aca="false">IF(D69="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B69" s="16"/>
-      <c r="C69" s="16"/>
-      <c r="D69" s="16"/>
-      <c r="E69" s="15"/>
-      <c r="F69" s="15"/>
-      <c r="G69" s="15"/>
-      <c r="H69" s="16"/>
-      <c r="I69" s="16"/>
-      <c r="J69" s="16"/>
-      <c r="K69" s="16"/>
-      <c r="L69" s="16"/>
-      <c r="M69" s="16"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="15" t="str">
+      <c r="B69" s="17"/>
+      <c r="C69" s="17"/>
+      <c r="D69" s="17"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+      <c r="G69" s="16"/>
+      <c r="H69" s="17"/>
+      <c r="I69" s="17"/>
+      <c r="J69" s="17"/>
+      <c r="K69" s="17"/>
+      <c r="L69" s="17"/>
+      <c r="M69" s="17"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="16" t="str">
         <f aca="false">IF(D70="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B70" s="16"/>
-      <c r="C70" s="16"/>
-      <c r="D70" s="16"/>
-      <c r="E70" s="15"/>
-      <c r="F70" s="15"/>
-      <c r="G70" s="15"/>
-      <c r="H70" s="16"/>
-      <c r="I70" s="16"/>
-      <c r="J70" s="16"/>
-      <c r="K70" s="16"/>
-      <c r="L70" s="16"/>
-      <c r="M70" s="16"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="15" t="str">
+      <c r="B70" s="17"/>
+      <c r="C70" s="17"/>
+      <c r="D70" s="17"/>
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+      <c r="G70" s="16"/>
+      <c r="H70" s="17"/>
+      <c r="I70" s="17"/>
+      <c r="J70" s="17"/>
+      <c r="K70" s="17"/>
+      <c r="L70" s="17"/>
+      <c r="M70" s="17"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="16" t="str">
         <f aca="false">IF(D71="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B71" s="16"/>
-      <c r="C71" s="16"/>
-      <c r="D71" s="16"/>
-      <c r="E71" s="15"/>
-      <c r="F71" s="15"/>
-      <c r="G71" s="15"/>
-      <c r="H71" s="16"/>
-      <c r="I71" s="16"/>
-      <c r="J71" s="16"/>
-      <c r="K71" s="16"/>
-      <c r="L71" s="16"/>
-      <c r="M71" s="16"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="15" t="str">
+      <c r="B71" s="17"/>
+      <c r="C71" s="17"/>
+      <c r="D71" s="17"/>
+      <c r="E71" s="16"/>
+      <c r="F71" s="16"/>
+      <c r="G71" s="16"/>
+      <c r="H71" s="17"/>
+      <c r="I71" s="17"/>
+      <c r="J71" s="17"/>
+      <c r="K71" s="17"/>
+      <c r="L71" s="17"/>
+      <c r="M71" s="17"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="16" t="str">
         <f aca="false">IF(D72="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B72" s="16"/>
-      <c r="C72" s="16"/>
-      <c r="D72" s="16"/>
-      <c r="E72" s="15"/>
-      <c r="F72" s="15"/>
-      <c r="G72" s="15"/>
-      <c r="H72" s="16"/>
-      <c r="I72" s="16"/>
-      <c r="J72" s="16"/>
-      <c r="K72" s="16"/>
-      <c r="L72" s="16"/>
-      <c r="M72" s="16"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="15" t="str">
+      <c r="B72" s="17"/>
+      <c r="C72" s="17"/>
+      <c r="D72" s="17"/>
+      <c r="E72" s="16"/>
+      <c r="F72" s="16"/>
+      <c r="G72" s="16"/>
+      <c r="H72" s="17"/>
+      <c r="I72" s="17"/>
+      <c r="J72" s="17"/>
+      <c r="K72" s="17"/>
+      <c r="L72" s="17"/>
+      <c r="M72" s="17"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="16" t="str">
         <f aca="false">IF(D73="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B73" s="16"/>
-      <c r="C73" s="16"/>
-      <c r="D73" s="16"/>
-      <c r="E73" s="15"/>
-      <c r="F73" s="15"/>
-      <c r="G73" s="15"/>
-      <c r="H73" s="16"/>
-      <c r="I73" s="16"/>
-      <c r="J73" s="16"/>
-      <c r="K73" s="16"/>
-      <c r="L73" s="16"/>
-      <c r="M73" s="16"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="15" t="str">
+      <c r="B73" s="17"/>
+      <c r="C73" s="17"/>
+      <c r="D73" s="17"/>
+      <c r="E73" s="16"/>
+      <c r="F73" s="16"/>
+      <c r="G73" s="16"/>
+      <c r="H73" s="17"/>
+      <c r="I73" s="17"/>
+      <c r="J73" s="17"/>
+      <c r="K73" s="17"/>
+      <c r="L73" s="17"/>
+      <c r="M73" s="17"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="16" t="str">
         <f aca="false">IF(D74="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B74" s="16"/>
-      <c r="C74" s="16"/>
-      <c r="D74" s="16"/>
-      <c r="E74" s="15"/>
-      <c r="F74" s="15"/>
-      <c r="G74" s="15"/>
-      <c r="H74" s="16"/>
-      <c r="I74" s="16"/>
-      <c r="J74" s="16"/>
-      <c r="K74" s="16"/>
-      <c r="L74" s="16"/>
-      <c r="M74" s="16"/>
+      <c r="B74" s="17"/>
+      <c r="C74" s="17"/>
+      <c r="D74" s="17"/>
+      <c r="E74" s="16"/>
+      <c r="F74" s="16"/>
+      <c r="G74" s="16"/>
+      <c r="H74" s="17"/>
+      <c r="I74" s="17"/>
+      <c r="J74" s="17"/>
+      <c r="K74" s="17"/>
+      <c r="L74" s="17"/>
+      <c r="M74" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M54"/>

</xml_diff>

<commit_message>
rules v1.4: chest/tumba overlay top overhangs 20 mm at the front
- Factory rule confirmed by the product owner (two real chests): overall
  depth = top depth, carcass depth = overall - 20; wardrobes stay flush.
- Inset panel 2 mm clearance recorded as technologist's choice (not a rule).
- HDF-in-groove formula (+14 / +16) recorded as an open question.
- Real-order fixtures: KR of both chests now match GibLab.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAoMGr6KDaXSM8LT5Nrkkp
</commit_message>
<xml_diff>
--- a/docs/Elvin_pytannia_tehnologu.xlsx
+++ b/docs/Elvin_pytannia_tehnologu.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="231">
   <si>
     <t xml:space="preserve">Elvin — питання технологу</t>
   </si>
@@ -679,6 +679,45 @@
   </si>
   <si>
     <t xml:space="preserve">Лишаємо KR08 0,8 мм; змінюється в 1 клік</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Накладна кришка комода/тумби глибша за корпус на 20 мм (виступ спереду)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Глибина кришки і корпусу.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комоди 1350 і 1800: 350/330, 500/480.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Так, стандарт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ХДФ у паз: лист = проріз + 14 мм по ширині і + 16 мм по висоті?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комоди 1350 і 1800: 1328 = 1314+14, 670 = 654+16; 1778 = 1764+14, 960 = 944+16.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Потрібне уточнення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вкладне дно/кришка на 2 мм вужчі за проріз?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Розмір DNO/KR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комоди: −2 мм; шафа 1500: рівно в проріз.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Залежить від технолога; Elvin рахує рівно в проріз</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
   </si>
 </sst>
 </file>
@@ -1355,7 +1394,7 @@
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A4)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито")</f>
@@ -1371,7 +1410,7 @@
       </c>
       <c r="F4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
@@ -1442,11 +1481,11 @@
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A7)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відкрито")</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відповідь отримано")</f>
@@ -1616,11 +1655,11 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">SUM(B4:B12)</f>
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">SUM(C4:C12)</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">SUM(D4:D12)</f>
@@ -1632,7 +1671,7 @@
       </c>
       <c r="F13" s="13" t="n">
         <f aca="false">SUM(F4:F12)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">SUM(G4:G12)</f>
@@ -1645,7 +1684,7 @@
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">IF(B13=0,0,F13/B13)</f>
-        <v>0.109090909090909</v>
+        <v>0.137931034482759</v>
       </c>
     </row>
   </sheetData>
@@ -3387,57 +3426,113 @@
       <c r="M56" s="17"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="16" t="str">
+      <c r="A57" s="16" t="n">
         <f aca="false">IF(D57="","",ROW()-1)</f>
-        <v/>
-      </c>
-      <c r="B57" s="17"/>
-      <c r="C57" s="17"/>
-      <c r="D57" s="17"/>
-      <c r="E57" s="16"/>
-      <c r="F57" s="16"/>
+        <v>56</v>
+      </c>
+      <c r="B57" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C57" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D57" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="E57" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="F57" s="16" t="s">
+        <v>220</v>
+      </c>
       <c r="G57" s="16"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17"/>
+      <c r="H57" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="I57" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="J57" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="K57" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="L57" s="17" t="s">
+        <v>24</v>
+      </c>
       <c r="M57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="16" t="str">
+      <c r="A58" s="16" t="n">
         <f aca="false">IF(D58="","",ROW()-1)</f>
-        <v/>
-      </c>
-      <c r="B58" s="17"/>
-      <c r="C58" s="17"/>
-      <c r="D58" s="17"/>
-      <c r="E58" s="16"/>
-      <c r="F58" s="16"/>
-      <c r="G58" s="16"/>
-      <c r="H58" s="17"/>
+        <v>57</v>
+      </c>
+      <c r="B58" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C58" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D58" s="17" t="s">
+        <v>223</v>
+      </c>
+      <c r="E58" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="F58" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="G58" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="H58" s="17" t="s">
+        <v>225</v>
+      </c>
       <c r="I58" s="17"/>
       <c r="J58" s="17"/>
       <c r="K58" s="17"/>
-      <c r="L58" s="17"/>
+      <c r="L58" s="17" t="s">
+        <v>21</v>
+      </c>
       <c r="M58" s="17"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="16" t="str">
+      <c r="A59" s="16" t="n">
         <f aca="false">IF(D59="","",ROW()-1)</f>
-        <v/>
-      </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="16"/>
-      <c r="F59" s="16"/>
+        <v>58</v>
+      </c>
+      <c r="B59" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C59" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="D59" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="E59" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="F59" s="16" t="s">
+        <v>228</v>
+      </c>
       <c r="G59" s="16"/>
-      <c r="H59" s="17"/>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17"/>
-      <c r="K59" s="17"/>
-      <c r="L59" s="17"/>
+      <c r="H59" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="I59" s="17" t="s">
+        <v>230</v>
+      </c>
+      <c r="J59" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="K59" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="L59" s="17" t="s">
+        <v>24</v>
+      </c>
       <c r="M59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
rules v1.5: factory standard for inner panels (exact fit, full depth)
Decision of the product owner to end 0/-1/-2 mm differences between
technologists: inset bottom/top, fixed and removable shelves and
partitions fit the opening exactly and use the full carcass depth with
overlay HDF. Earlier real-order deviations are kept as technologist
variants in the fixtures, not as Engine errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAoMGr6KDaXSM8LT5Nrkkp
</commit_message>
<xml_diff>
--- a/docs/Elvin_pytannia_tehnologu.xlsx
+++ b/docs/Elvin_pytannia_tehnologu.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="237">
   <si>
     <t xml:space="preserve">Elvin — питання технологу</t>
   </si>
@@ -255,6 +255,18 @@
     <t xml:space="preserve">Стандарт: глибина полиці = глибина корпусу.</t>
   </si>
   <si>
+    <t xml:space="preserve">Стандарт: на всю глибину корпусу (при накладній ХДФ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Користувач (чат)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.10.2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Полиці кріпляться на конфірмати (нерухомі) чи стоять на полицетримачах (знімні)? Як це позначається?</t>
   </si>
   <si>
@@ -621,12 +633,6 @@
     <t xml:space="preserve">3 / 3 / 2 / 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Користувач (чат)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.10.2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Між фасадами 4 мм — за реальним замовленням (GibLab), підтверджено 16.10.2026</t>
   </si>
   <si>
@@ -714,10 +720,22 @@
     <t xml:space="preserve">Комоди: −2 мм; шафа 1500: рівно в проріз.</t>
   </si>
   <si>
-    <t xml:space="preserve">Залежить від технолога; Elvin рахує рівно в проріз</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0</t>
+    <t xml:space="preserve">Стандарт фабрики: рівно в проріз (без відступу)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Єдиний стандарт для внутрішніх деталей (дно, кришка, полиці, стійки): відступи по довжині й глибині?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Однаковий результат у всіх технологів.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">У замовленнях траплялось 0, −1, −2 мм.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рівно в проріз і на всю глибину; знімні полиці — так само</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 / 0</t>
   </si>
 </sst>
 </file>
@@ -1394,7 +1412,7 @@
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIF(Питання!$B$2:$B$200,A4)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито")</f>
@@ -1410,7 +1428,7 @@
       </c>
       <c r="F4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
@@ -1427,7 +1445,7 @@
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Відкрито")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Відповідь отримано")</f>
@@ -1439,7 +1457,7 @@
       </c>
       <c r="F5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A5,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
@@ -1655,11 +1673,11 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">SUM(B4:B12)</f>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">SUM(C4:C12)</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">SUM(D4:D12)</f>
@@ -1671,7 +1689,7 @@
       </c>
       <c r="F13" s="13" t="n">
         <f aca="false">SUM(F4:F12)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">SUM(G4:G12)</f>
@@ -1684,7 +1702,7 @@
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">IF(B13=0,0,F13/B13)</f>
-        <v>0.137931034482759</v>
+        <v>0.169491525423729</v>
       </c>
     </row>
   </sheetData>
@@ -1991,12 +2009,20 @@
         <v>75</v>
       </c>
       <c r="G9" s="16"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
+      <c r="H9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="J9" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>79</v>
+      </c>
       <c r="L9" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="M9" s="17"/>
     </row>
@@ -2011,16 +2037,16 @@
         <v>51</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F10" s="16" t="s">
         <v>64</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -2042,10 +2068,10 @@
         <v>51</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F11" s="16" t="s">
         <v>64</v>
@@ -2071,10 +2097,10 @@
         <v>58</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F12" s="16" t="s">
         <v>64</v>
@@ -2100,13 +2126,13 @@
         <v>51</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="17"/>
@@ -2129,13 +2155,13 @@
         <v>51</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G14" s="16"/>
       <c r="H14" s="17"/>
@@ -2158,10 +2184,10 @@
         <v>58</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F15" s="16" t="s">
         <v>64</v>
@@ -2187,18 +2213,18 @@
         <v>46</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G16" s="16"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
@@ -2206,7 +2232,7 @@
         <v>21</v>
       </c>
       <c r="M16" s="18" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2220,10 +2246,10 @@
         <v>46</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F17" s="16" t="s">
         <v>64</v>
@@ -2249,16 +2275,16 @@
         <v>51</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -2280,13 +2306,13 @@
         <v>51</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="17"/>
@@ -2309,13 +2335,13 @@
         <v>51</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G20" s="16"/>
       <c r="H20" s="17"/>
@@ -2338,16 +2364,16 @@
         <v>51</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H21" s="17"/>
       <c r="I21" s="17"/>
@@ -2369,13 +2395,13 @@
         <v>51</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="17"/>
@@ -2398,10 +2424,10 @@
         <v>51</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F23" s="16" t="s">
         <v>64</v>
@@ -2427,13 +2453,13 @@
         <v>46</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="G24" s="16"/>
       <c r="H24" s="17"/>
@@ -2456,18 +2482,18 @@
         <v>51</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="17"/>
       <c r="I25" s="17" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
@@ -2475,7 +2501,7 @@
         <v>21</v>
       </c>
       <c r="M25" s="18" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2489,13 +2515,13 @@
         <v>51</v>
       </c>
       <c r="D26" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="E26" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="E26" s="16" t="s">
-        <v>121</v>
-      </c>
       <c r="F26" s="16" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G26" s="16"/>
       <c r="H26" s="17"/>
@@ -2518,13 +2544,13 @@
         <v>51</v>
       </c>
       <c r="D27" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="E27" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="F27" s="16" t="s">
         <v>126</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="F27" s="16" t="s">
-        <v>122</v>
       </c>
       <c r="G27" s="16"/>
       <c r="H27" s="17"/>
@@ -2547,13 +2573,13 @@
         <v>46</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E28" s="16" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G28" s="16"/>
       <c r="H28" s="17"/>
@@ -2576,13 +2602,13 @@
         <v>58</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="17"/>
@@ -2605,16 +2631,16 @@
         <v>51</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
@@ -2636,13 +2662,13 @@
         <v>51</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G31" s="16"/>
       <c r="H31" s="17"/>
@@ -2665,13 +2691,13 @@
         <v>51</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G32" s="16"/>
       <c r="H32" s="17"/>
@@ -2694,10 +2720,10 @@
         <v>58</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F33" s="16" t="s">
         <v>64</v>
@@ -2723,13 +2749,13 @@
         <v>51</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="G34" s="16"/>
       <c r="H34" s="17"/>
@@ -2752,10 +2778,10 @@
         <v>58</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F35" s="16" t="s">
         <v>64</v>
@@ -2781,13 +2807,13 @@
         <v>51</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E36" s="16" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G36" s="16"/>
       <c r="H36" s="17"/>
@@ -2810,16 +2836,16 @@
         <v>51</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H37" s="17"/>
       <c r="I37" s="17"/>
@@ -2841,16 +2867,16 @@
         <v>51</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E38" s="16" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
@@ -2872,16 +2898,16 @@
         <v>51</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E39" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="F39" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="G39" s="16" t="s">
         <v>158</v>
-      </c>
-      <c r="F39" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="G39" s="16" t="s">
-        <v>154</v>
       </c>
       <c r="H39" s="17"/>
       <c r="I39" s="17"/>
@@ -2903,13 +2929,13 @@
         <v>58</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E40" s="16" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G40" s="16"/>
       <c r="H40" s="17"/>
@@ -2932,18 +2958,18 @@
         <v>51</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="17"/>
       <c r="I41" s="17" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
@@ -2951,7 +2977,7 @@
         <v>21</v>
       </c>
       <c r="M41" s="18" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2965,13 +2991,13 @@
         <v>58</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="G42" s="16"/>
       <c r="H42" s="17"/>
@@ -2994,10 +3020,10 @@
         <v>58</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E43" s="16" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F43" s="16" t="s">
         <v>64</v>
@@ -3023,16 +3049,16 @@
         <v>51</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
@@ -3054,13 +3080,13 @@
         <v>58</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="17"/>
@@ -3083,13 +3109,13 @@
         <v>58</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="G46" s="16"/>
       <c r="H46" s="17"/>
@@ -3112,13 +3138,13 @@
         <v>51</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="F47" s="16" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="G47" s="16"/>
       <c r="H47" s="17"/>
@@ -3141,13 +3167,13 @@
         <v>51</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E48" s="16" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F48" s="16" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="G48" s="16"/>
       <c r="H48" s="17"/>
@@ -3170,13 +3196,13 @@
         <v>58</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="G49" s="16"/>
       <c r="H49" s="17"/>
@@ -3199,13 +3225,13 @@
         <v>58</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E50" s="16" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="G50" s="16"/>
       <c r="H50" s="17"/>
@@ -3228,30 +3254,30 @@
         <v>46</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="F51" s="16"/>
       <c r="G51" s="16"/>
       <c r="H51" s="17" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="I51" s="17" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="J51" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K51" s="17" t="s">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="L51" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M51" s="17" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3265,24 +3291,24 @@
         <v>46</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E52" s="16" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F52" s="16"/>
       <c r="G52" s="16"/>
       <c r="H52" s="17" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="I52" s="17" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="J52" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K52" s="17" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="L52" s="17" t="s">
         <v>24</v>
@@ -3300,22 +3326,22 @@
         <v>51</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F53" s="16"/>
       <c r="G53" s="16"/>
       <c r="H53" s="17" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I53" s="17"/>
       <c r="J53" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K53" s="17" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="L53" s="17" t="s">
         <v>24</v>
@@ -3333,22 +3359,22 @@
         <v>51</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E54" s="16" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F54" s="16"/>
       <c r="G54" s="16"/>
       <c r="H54" s="17" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I54" s="17"/>
       <c r="J54" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K54" s="17" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="L54" s="17" t="s">
         <v>24</v>
@@ -3367,22 +3393,22 @@
         <v>51</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E55" s="16" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F55" s="16"/>
       <c r="G55" s="16"/>
       <c r="H55" s="17" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I55" s="17"/>
       <c r="J55" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K55" s="17" t="s">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="L55" s="17" t="s">
         <v>24</v>
@@ -3401,24 +3427,24 @@
         <v>58</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E56" s="16" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F56" s="16" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G56" s="16"/>
       <c r="H56" s="17" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I56" s="17"/>
       <c r="J56" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K56" s="17" t="s">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="L56" s="17" t="s">
         <v>24</v>
@@ -3437,26 +3463,26 @@
         <v>46</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E57" s="16" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F57" s="16" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G57" s="16"/>
       <c r="H57" s="17" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="I57" s="17" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J57" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K57" s="17" t="s">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="L57" s="17" t="s">
         <v>24</v>
@@ -3475,19 +3501,19 @@
         <v>51</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E58" s="16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F58" s="16" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G58" s="16" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H58" s="17" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I58" s="17"/>
       <c r="J58" s="17"/>
@@ -3509,26 +3535,26 @@
         <v>58</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G59" s="16"/>
       <c r="H59" s="17" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="I59" s="17" t="s">
-        <v>230</v>
+        <v>77</v>
       </c>
       <c r="J59" s="17" t="s">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="K59" s="17" t="s">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="L59" s="17" t="s">
         <v>24</v>
@@ -3536,21 +3562,41 @@
       <c r="M59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="16" t="str">
+      <c r="A60" s="16" t="n">
         <f aca="false">IF(D60="","",ROW()-1)</f>
-        <v/>
-      </c>
-      <c r="B60" s="17"/>
-      <c r="C60" s="17"/>
-      <c r="D60" s="17"/>
-      <c r="E60" s="16"/>
-      <c r="F60" s="16"/>
+        <v>59</v>
+      </c>
+      <c r="B60" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C60" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D60" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="E60" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="F60" s="16" t="s">
+        <v>234</v>
+      </c>
       <c r="G60" s="16"/>
-      <c r="H60" s="17"/>
-      <c r="I60" s="17"/>
-      <c r="J60" s="17"/>
-      <c r="K60" s="17"/>
-      <c r="L60" s="17"/>
+      <c r="H60" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="I60" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="J60" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K60" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L60" s="17" t="s">
+        <v>24</v>
+      </c>
       <c r="M60" s="17"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
rules v1.6: groove standard (14 mm from back, 4x9) and DSP 18 mm only
- Groove: shelves, partitions and an inset top stop 18 mm (14 + 4) before
  the back; sides, bottom and overlay top keep full depth. No question
  about the groove offset any more. Matches the real top box (KR 804x510).
- Factory uses only DSP 18 mm; another thickness gives a warning.
- Fixtures: groove variants made before the standard kept as variants.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAoMGr6KDaXSM8LT5Nrkkp
</commit_message>
<xml_diff>
--- a/docs/Elvin_pytannia_tehnologu.xlsx
+++ b/docs/Elvin_pytannia_tehnologu.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="244">
   <si>
     <t xml:space="preserve">Elvin — питання технологу</t>
   </si>
@@ -213,6 +213,18 @@
     <t xml:space="preserve">Статус ASK: шари 18+18, клей ≈1 мм.</t>
   </si>
   <si>
+    <t xml:space="preserve">Фабрика використовує лише ДСП 18; 37 мм = два листи по 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18+18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Користувач (чат)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.10.2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Розміри секцій на кресленнях зазвичай проставлені у світлі (між деталями), по осях чи зовнішні?</t>
   </si>
   <si>
@@ -261,9 +273,6 @@
     <t xml:space="preserve">0</t>
   </si>
   <si>
-    <t xml:space="preserve">Користувач (чат)</t>
-  </si>
-  <si>
     <t xml:space="preserve">16.10.2026</t>
   </si>
   <si>
@@ -384,6 +393,12 @@
     <t xml:space="preserve">Дозволено 5–20 мм.</t>
   </si>
   <si>
+    <t xml:space="preserve">14 мм від заднього краю; паз 4 × 9 мм</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14</t>
+  </si>
+  <si>
     <t xml:space="preserve">ХДФ у паз: максимальний розмір листа?</t>
   </si>
   <si>
@@ -550,6 +565,12 @@
   </si>
   <si>
     <t xml:space="preserve">Стандарт ДСП 18, МДФ — за проєктом.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ДСП 18 мм (фабрика використовує лише ДСП 18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18</t>
   </si>
   <si>
     <t xml:space="preserve">Петлі та ручки: чи має Elvin додавати їх і свердління під них у BAZIS? Кількість петель за висотою фасаду?</t>
@@ -1416,7 +1437,7 @@
       </c>
       <c r="C4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відповідь отримано")</f>
@@ -1428,7 +1449,7 @@
       </c>
       <c r="F4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A4,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
@@ -1503,7 +1524,7 @@
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відкрито")</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відповідь отримано")</f>
@@ -1515,7 +1536,7 @@
       </c>
       <c r="F7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
@@ -1590,7 +1611,7 @@
       </c>
       <c r="C10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Відкрито")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Відповідь отримано")</f>
@@ -1602,7 +1623,7 @@
       </c>
       <c r="F10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A10,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
@@ -1677,7 +1698,7 @@
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">SUM(C4:C12)</f>
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">SUM(D4:D12)</f>
@@ -1689,7 +1710,7 @@
       </c>
       <c r="F13" s="13" t="n">
         <f aca="false">SUM(F4:F12)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">SUM(G4:G12)</f>
@@ -1702,7 +1723,7 @@
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">IF(B13=0,0,F13/B13)</f>
-        <v>0.169491525423729</v>
+        <v>0.220338983050847</v>
       </c>
     </row>
   </sheetData>
@@ -1889,12 +1910,20 @@
         <v>61</v>
       </c>
       <c r="G5" s="16"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
+      <c r="H5" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>65</v>
+      </c>
       <c r="L5" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="M5" s="17"/>
     </row>
@@ -1909,16 +1938,16 @@
         <v>46</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
@@ -1940,13 +1969,13 @@
         <v>46</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="17"/>
@@ -1969,16 +1998,16 @@
         <v>46</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
@@ -2000,26 +2029,26 @@
         <v>51</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="17" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I9" s="17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K9" s="17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L9" s="17" t="s">
         <v>24</v>
@@ -2037,16 +2066,16 @@
         <v>51</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -2068,13 +2097,13 @@
         <v>51</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="17"/>
@@ -2097,13 +2126,13 @@
         <v>58</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="17"/>
@@ -2126,13 +2155,13 @@
         <v>51</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="17"/>
@@ -2155,13 +2184,13 @@
         <v>51</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G14" s="16"/>
       <c r="H14" s="17"/>
@@ -2184,13 +2213,13 @@
         <v>58</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="17"/>
@@ -2213,18 +2242,18 @@
         <v>46</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G16" s="16"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
@@ -2232,7 +2261,7 @@
         <v>21</v>
       </c>
       <c r="M16" s="18" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2246,13 +2275,13 @@
         <v>46</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="17"/>
@@ -2275,16 +2304,16 @@
         <v>51</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -2306,13 +2335,13 @@
         <v>51</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="17"/>
@@ -2335,13 +2364,13 @@
         <v>51</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G20" s="16"/>
       <c r="H20" s="17"/>
@@ -2364,16 +2393,16 @@
         <v>51</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H21" s="17"/>
       <c r="I21" s="17"/>
@@ -2395,21 +2424,29 @@
         <v>51</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G22" s="16"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
+      <c r="H22" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="I22" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="J22" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="K22" s="17" t="s">
+        <v>65</v>
+      </c>
       <c r="L22" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="M22" s="17"/>
     </row>
@@ -2424,13 +2461,13 @@
         <v>51</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G23" s="16"/>
       <c r="H23" s="17"/>
@@ -2453,13 +2490,13 @@
         <v>46</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="G24" s="16"/>
       <c r="H24" s="17"/>
@@ -2482,18 +2519,18 @@
         <v>51</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="17"/>
       <c r="I25" s="17" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
@@ -2501,7 +2538,7 @@
         <v>21</v>
       </c>
       <c r="M25" s="18" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2515,13 +2552,13 @@
         <v>51</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="G26" s="16"/>
       <c r="H26" s="17"/>
@@ -2544,13 +2581,13 @@
         <v>51</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="G27" s="16"/>
       <c r="H27" s="17"/>
@@ -2573,13 +2610,13 @@
         <v>46</v>
       </c>
       <c r="D28" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" s="16" t="s">
         <v>131</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>132</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>126</v>
       </c>
       <c r="G28" s="16"/>
       <c r="H28" s="17"/>
@@ -2602,13 +2639,13 @@
         <v>58</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="17"/>
@@ -2631,16 +2668,16 @@
         <v>51</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
@@ -2662,13 +2699,13 @@
         <v>51</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G31" s="16"/>
       <c r="H31" s="17"/>
@@ -2691,13 +2728,13 @@
         <v>51</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="G32" s="16"/>
       <c r="H32" s="17"/>
@@ -2720,13 +2757,13 @@
         <v>58</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="17"/>
@@ -2749,13 +2786,13 @@
         <v>51</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="G34" s="16"/>
       <c r="H34" s="17"/>
@@ -2778,13 +2815,13 @@
         <v>58</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G35" s="16"/>
       <c r="H35" s="17"/>
@@ -2807,13 +2844,13 @@
         <v>51</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E36" s="16" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G36" s="16"/>
       <c r="H36" s="17"/>
@@ -2836,16 +2873,16 @@
         <v>51</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H37" s="17"/>
       <c r="I37" s="17"/>
@@ -2867,16 +2904,16 @@
         <v>51</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="E38" s="16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
@@ -2898,16 +2935,16 @@
         <v>51</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F39" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="G39" s="16" t="s">
         <v>163</v>
-      </c>
-      <c r="G39" s="16" t="s">
-        <v>158</v>
       </c>
       <c r="H39" s="17"/>
       <c r="I39" s="17"/>
@@ -2929,13 +2966,13 @@
         <v>58</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="E40" s="16" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="G40" s="16"/>
       <c r="H40" s="17"/>
@@ -2958,18 +2995,18 @@
         <v>51</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="17"/>
       <c r="I41" s="17" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
@@ -2977,7 +3014,7 @@
         <v>21</v>
       </c>
       <c r="M41" s="18" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2991,21 +3028,29 @@
         <v>58</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="G42" s="16"/>
-      <c r="H42" s="17"/>
-      <c r="I42" s="17"/>
-      <c r="J42" s="17"/>
-      <c r="K42" s="17"/>
+      <c r="H42" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="I42" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="J42" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="K42" s="17" t="s">
+        <v>65</v>
+      </c>
       <c r="L42" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="M42" s="17"/>
     </row>
@@ -3020,13 +3065,13 @@
         <v>58</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="E43" s="16" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G43" s="16"/>
       <c r="H43" s="17"/>
@@ -3049,16 +3094,16 @@
         <v>51</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
@@ -3080,13 +3125,13 @@
         <v>58</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="17"/>
@@ -3109,13 +3154,13 @@
         <v>58</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="G46" s="16"/>
       <c r="H46" s="17"/>
@@ -3138,13 +3183,13 @@
         <v>51</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="F47" s="16" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="G47" s="16"/>
       <c r="H47" s="17"/>
@@ -3167,13 +3212,13 @@
         <v>51</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="E48" s="16" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F48" s="16" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="G48" s="16"/>
       <c r="H48" s="17"/>
@@ -3196,13 +3241,13 @@
         <v>58</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="G49" s="16"/>
       <c r="H49" s="17"/>
@@ -3225,13 +3270,13 @@
         <v>58</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="E50" s="16" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="G50" s="16"/>
       <c r="H50" s="17"/>
@@ -3254,30 +3299,30 @@
         <v>46</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="F51" s="16"/>
       <c r="G51" s="16"/>
       <c r="H51" s="17" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="I51" s="17" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="J51" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K51" s="17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L51" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M51" s="17" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3291,24 +3336,24 @@
         <v>46</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="E52" s="16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F52" s="16"/>
       <c r="G52" s="16"/>
       <c r="H52" s="17" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="I52" s="17" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="J52" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K52" s="17" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="L52" s="17" t="s">
         <v>24</v>
@@ -3326,22 +3371,22 @@
         <v>51</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="F53" s="16"/>
       <c r="G53" s="16"/>
       <c r="H53" s="17" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="I53" s="17"/>
       <c r="J53" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K53" s="17" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="L53" s="17" t="s">
         <v>24</v>
@@ -3359,22 +3404,22 @@
         <v>51</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="E54" s="16" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="F54" s="16"/>
       <c r="G54" s="16"/>
       <c r="H54" s="17" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="I54" s="17"/>
       <c r="J54" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K54" s="17" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="L54" s="17" t="s">
         <v>24</v>
@@ -3393,22 +3438,22 @@
         <v>51</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="E55" s="16" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="F55" s="16"/>
       <c r="G55" s="16"/>
       <c r="H55" s="17" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="I55" s="17"/>
       <c r="J55" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K55" s="17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L55" s="17" t="s">
         <v>24</v>
@@ -3427,24 +3472,24 @@
         <v>58</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="E56" s="16" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="F56" s="16" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="G56" s="16"/>
       <c r="H56" s="17" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="I56" s="17"/>
       <c r="J56" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K56" s="17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L56" s="17" t="s">
         <v>24</v>
@@ -3463,26 +3508,26 @@
         <v>46</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="E57" s="16" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="F57" s="16" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="G57" s="16"/>
       <c r="H57" s="17" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="I57" s="17" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="J57" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K57" s="17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L57" s="17" t="s">
         <v>24</v>
@@ -3501,19 +3546,19 @@
         <v>51</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E58" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F58" s="16" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="G58" s="16" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H58" s="17" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="I58" s="17"/>
       <c r="J58" s="17"/>
@@ -3535,26 +3580,26 @@
         <v>58</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="G59" s="16"/>
       <c r="H59" s="17" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="I59" s="17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="J59" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K59" s="17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L59" s="17" t="s">
         <v>24</v>
@@ -3573,26 +3618,26 @@
         <v>46</v>
       </c>
       <c r="D60" s="17" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="F60" s="16" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="G60" s="16"/>
       <c r="H60" s="17" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="I60" s="17" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="J60" s="17" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K60" s="17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L60" s="17" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
rules v1.7: DSP 18 mm and glued 37 mm (18 + 18 + 1 mm glue)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAoMGr6KDaXSM8LT5Nrkkp
</commit_message>
<xml_diff>
--- a/docs/Elvin_pytannia_tehnologu.xlsx
+++ b/docs/Elvin_pytannia_tehnologu.xlsx
@@ -213,10 +213,10 @@
     <t xml:space="preserve">Статус ASK: шари 18+18, клей ≈1 мм.</t>
   </si>
   <si>
-    <t xml:space="preserve">Фабрика використовує лише ДСП 18; 37 мм = два листи по 18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18+18</t>
+    <t xml:space="preserve">ДСП 18 або склейка 37 мм (18 + 18 + 1 мм клею)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 / 37</t>
   </si>
   <si>
     <t xml:space="preserve">Користувач (чат)</t>
@@ -567,7 +567,7 @@
     <t xml:space="preserve">Стандарт ДСП 18, МДФ — за проєктом.</t>
   </si>
   <si>
-    <t xml:space="preserve">ДСП 18 мм (фабрика використовує лише ДСП 18)</t>
+    <t xml:space="preserve">ДСП 18 мм (фабрика використовує ДСП 18 і склейку 37 мм)</t>
   </si>
   <si>
     <t xml:space="preserve">18</t>

</xml_diff>

<commit_message>
rules v1.8: HDF in groove is built (groove in sides and bottom)
- Groove in left side, right side and bottom; HDF slides in from the top
  behind an inset top. Sheet = opening + 16 (8 mm into each groove),
  bottom edge 8 mm into the bottom groove, top 1 mm below the carcass top.
- Engine builds the TYL part; geometry check allows it to sit in the
  grooves; BAZIS code includes it (front panel).
- Overlay top with groove is asked, not guessed.
- Real top box 840 now matches GibLab including HDF 820x489.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAoMGr6KDaXSM8LT5Nrkkp
</commit_message>
<xml_diff>
--- a/docs/Elvin_pytannia_tehnologu.xlsx
+++ b/docs/Elvin_pytannia_tehnologu.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="247">
   <si>
     <t xml:space="preserve">Elvin — питання технологу</t>
   </si>
@@ -384,6 +384,12 @@
     <t xml:space="preserve">Паз у кришці / Під кришку</t>
   </si>
   <si>
+    <t xml:space="preserve">Паз лише з 3 боків (ліва, права, дно); ХДФ вставляється зверху за вкладну кришку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Відкрито: як при накладній кришці (у GibLab траплялось KR_PAZ)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ХДФ у паз: стандартний відступ паза від заднього краю?</t>
   </si>
   <si>
@@ -729,7 +735,10 @@
     <t xml:space="preserve">Комоди 1350 і 1800: 1328 = 1314+14, 670 = 654+16; 1778 = 1764+14, 960 = 944+16.</t>
   </si>
   <si>
-    <t xml:space="preserve">Потрібне уточнення</t>
+    <t xml:space="preserve">Паз у лівій, правій боковині і дні; ХДФ = проріз + 16 (по 8 мм у паз)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+16</t>
   </si>
   <si>
     <t xml:space="preserve">Вкладне дно/кришка на 2 мм вужчі за проріз?</t>
@@ -1524,7 +1533,7 @@
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відкрито")</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відповідь отримано")</f>
@@ -1536,7 +1545,7 @@
       </c>
       <c r="F7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Внесено в Elvin")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G7" s="11" t="n">
         <f aca="false">COUNTIFS(Питання!$B$2:$B$200,A7,Питання!$L$2:$L$200,"Відкрито",Питання!$C$2:$C$200,"Високий")</f>
@@ -1698,7 +1707,7 @@
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">SUM(C4:C12)</f>
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">SUM(D4:D12)</f>
@@ -1710,7 +1719,7 @@
       </c>
       <c r="F13" s="13" t="n">
         <f aca="false">SUM(F4:F12)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">SUM(G4:G12)</f>
@@ -1723,7 +1732,7 @@
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">IF(B13=0,0,F13/B13)</f>
-        <v>0.220338983050847</v>
+        <v>0.254237288135593</v>
       </c>
     </row>
   </sheetData>
@@ -2404,14 +2413,22 @@
       <c r="G21" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="H21" s="17"/>
+      <c r="H21" s="17" t="s">
+        <v>119</v>
+      </c>
       <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
+      <c r="J21" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>65</v>
+      </c>
       <c r="L21" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="M21" s="17"/>
+        <v>24</v>
+      </c>
+      <c r="M21" s="17" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="n">
@@ -2424,20 +2441,20 @@
         <v>51</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="17" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="J22" s="17" t="s">
         <v>64</v>
@@ -2461,10 +2478,10 @@
         <v>51</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F23" s="16" t="s">
         <v>68</v>
@@ -2490,13 +2507,13 @@
         <v>46</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G24" s="16"/>
       <c r="H24" s="17"/>
@@ -2519,18 +2536,18 @@
         <v>51</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="17"/>
       <c r="I25" s="17" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
@@ -2538,7 +2555,7 @@
         <v>21</v>
       </c>
       <c r="M25" s="18" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2552,13 +2569,13 @@
         <v>51</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G26" s="16"/>
       <c r="H26" s="17"/>
@@ -2581,13 +2598,13 @@
         <v>51</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E27" s="16" t="s">
         <v>99</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G27" s="16"/>
       <c r="H27" s="17"/>
@@ -2610,13 +2627,13 @@
         <v>46</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E28" s="16" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G28" s="16"/>
       <c r="H28" s="17"/>
@@ -2639,13 +2656,13 @@
         <v>58</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="17"/>
@@ -2668,16 +2685,16 @@
         <v>51</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
@@ -2699,13 +2716,13 @@
         <v>51</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G31" s="16"/>
       <c r="H31" s="17"/>
@@ -2728,13 +2745,13 @@
         <v>51</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G32" s="16"/>
       <c r="H32" s="17"/>
@@ -2757,7 +2774,7 @@
         <v>58</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E33" s="16" t="s">
         <v>94</v>
@@ -2786,13 +2803,13 @@
         <v>51</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G34" s="16"/>
       <c r="H34" s="17"/>
@@ -2815,10 +2832,10 @@
         <v>58</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F35" s="16" t="s">
         <v>68</v>
@@ -2844,13 +2861,13 @@
         <v>51</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E36" s="16" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G36" s="16"/>
       <c r="H36" s="17"/>
@@ -2873,16 +2890,16 @@
         <v>51</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H37" s="17"/>
       <c r="I37" s="17"/>
@@ -2904,16 +2921,16 @@
         <v>51</v>
       </c>
       <c r="D38" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="E38" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="F38" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="E38" s="16" t="s">
+      <c r="G38" s="16" t="s">
         <v>165</v>
-      </c>
-      <c r="F38" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="G38" s="16" t="s">
-        <v>163</v>
       </c>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
@@ -2935,16 +2952,16 @@
         <v>51</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H39" s="17"/>
       <c r="I39" s="17"/>
@@ -2966,13 +2983,13 @@
         <v>58</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E40" s="16" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G40" s="16"/>
       <c r="H40" s="17"/>
@@ -2995,18 +3012,18 @@
         <v>51</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="17"/>
       <c r="I41" s="17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
@@ -3014,7 +3031,7 @@
         <v>21</v>
       </c>
       <c r="M41" s="18" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3028,20 +3045,20 @@
         <v>58</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G42" s="16"/>
       <c r="H42" s="17" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I42" s="17" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J42" s="17" t="s">
         <v>64</v>
@@ -3065,10 +3082,10 @@
         <v>58</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E43" s="16" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F43" s="16" t="s">
         <v>68</v>
@@ -3094,16 +3111,16 @@
         <v>51</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
@@ -3125,13 +3142,13 @@
         <v>58</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="17"/>
@@ -3154,13 +3171,13 @@
         <v>58</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G46" s="16"/>
       <c r="H46" s="17"/>
@@ -3183,13 +3200,13 @@
         <v>51</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F47" s="16" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G47" s="16"/>
       <c r="H47" s="17"/>
@@ -3212,13 +3229,13 @@
         <v>51</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E48" s="16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F48" s="16" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G48" s="16"/>
       <c r="H48" s="17"/>
@@ -3241,13 +3258,13 @@
         <v>58</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G49" s="16"/>
       <c r="H49" s="17"/>
@@ -3270,13 +3287,13 @@
         <v>58</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E50" s="16" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G50" s="16"/>
       <c r="H50" s="17"/>
@@ -3299,18 +3316,18 @@
         <v>46</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F51" s="16"/>
       <c r="G51" s="16"/>
       <c r="H51" s="17" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I51" s="17" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J51" s="17" t="s">
         <v>64</v>
@@ -3322,7 +3339,7 @@
         <v>24</v>
       </c>
       <c r="M51" s="17" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3336,24 +3353,24 @@
         <v>46</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E52" s="16" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F52" s="16"/>
       <c r="G52" s="16"/>
       <c r="H52" s="17" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I52" s="17" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="J52" s="17" t="s">
         <v>64</v>
       </c>
       <c r="K52" s="17" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L52" s="17" t="s">
         <v>24</v>
@@ -3371,22 +3388,22 @@
         <v>51</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F53" s="16"/>
       <c r="G53" s="16"/>
       <c r="H53" s="17" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="I53" s="17"/>
       <c r="J53" s="17" t="s">
         <v>64</v>
       </c>
       <c r="K53" s="17" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L53" s="17" t="s">
         <v>24</v>
@@ -3404,22 +3421,22 @@
         <v>51</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E54" s="16" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F54" s="16"/>
       <c r="G54" s="16"/>
       <c r="H54" s="17" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I54" s="17"/>
       <c r="J54" s="17" t="s">
         <v>64</v>
       </c>
       <c r="K54" s="17" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L54" s="17" t="s">
         <v>24</v>
@@ -3438,15 +3455,15 @@
         <v>51</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E55" s="16" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F55" s="16"/>
       <c r="G55" s="16"/>
       <c r="H55" s="17" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I55" s="17"/>
       <c r="J55" s="17" t="s">
@@ -3472,17 +3489,17 @@
         <v>58</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E56" s="16" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F56" s="16" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G56" s="16"/>
       <c r="H56" s="17" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="I56" s="17"/>
       <c r="J56" s="17" t="s">
@@ -3508,20 +3525,20 @@
         <v>46</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E57" s="16" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F57" s="16" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G57" s="16"/>
       <c r="H57" s="17" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="I57" s="17" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J57" s="17" t="s">
         <v>64</v>
@@ -3546,25 +3563,31 @@
         <v>51</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E58" s="16" t="s">
         <v>113</v>
       </c>
       <c r="F58" s="16" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="G58" s="16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H58" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="I58" s="17"/>
-      <c r="J58" s="17"/>
-      <c r="K58" s="17"/>
+        <v>236</v>
+      </c>
+      <c r="I58" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="J58" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="K58" s="17" t="s">
+        <v>65</v>
+      </c>
       <c r="L58" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="M58" s="17"/>
     </row>
@@ -3580,17 +3603,17 @@
         <v>58</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="G59" s="16"/>
       <c r="H59" s="17" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="I59" s="17" t="s">
         <v>81</v>
@@ -3618,20 +3641,20 @@
         <v>46</v>
       </c>
       <c r="D60" s="17" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="F60" s="16" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="G60" s="16"/>
       <c r="H60" s="17" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I60" s="17" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="J60" s="17" t="s">
         <v>64</v>

</xml_diff>